<commit_message>
Box 47's caption says more than, not more then
</commit_message>
<xml_diff>
--- a/app/templates/se/Financialaccounts.xlsx
+++ b/app/templates/se/Financialaccounts.xlsx
@@ -16509,8 +16509,10 @@
         <v>47</v>
       </c>
       <c r="B126" s="220"/>
-      <c r="C126" s="227" t="s">
-        <v>214</v>
+      <c r="C126" s="227" t="inlineStr">
+        <is>
+          <t>Net profit - if your business income is more than your</t>
+        </is>
       </c>
       <c r="D126" s="227"/>
       <c r="E126" s="227"/>

</xml_diff>

<commit_message>
Clear the empty boxes the removed captions left behind
Boxes 66, 67, 69 and 70 are not in use, and box 11 went with them, so the
date and money fields those boxes used to fill now belong to nothing. Their
borders come off on both the return and the Business Details input beside it,
leaving the form's own 'not in use' note with nothing to fill in under it.
</commit_message>
<xml_diff>
--- a/app/templates/se/Financialaccounts.xlsx
+++ b/app/templates/se/Financialaccounts.xlsx
@@ -7703,7 +7703,7 @@
     <row r="45" spans="1:23" ht="18" x14ac:dyDescent="0.2">
       <c r="A45" s="185"/>
       <c r="B45" s="181"/>
-      <c r="C45" s="196"/>
+      <c r="C45" s="181"/>
       <c r="D45" s="181"/>
       <c r="E45" s="181"/>
       <c r="F45" s="181"/>
@@ -14095,7 +14095,7 @@
     <row r="48" spans="1:23" ht="14" x14ac:dyDescent="0.15">
       <c r="A48" s="240"/>
       <c r="B48" s="220"/>
-      <c r="C48" s="272"/>
+      <c r="C48" s="227"/>
       <c r="D48" s="220"/>
       <c r="E48" s="220"/>
       <c r="F48" s="220"/>
@@ -18426,10 +18426,10 @@
     <row r="187" spans="1:23" ht="14" x14ac:dyDescent="0.15">
       <c r="A187" s="255"/>
       <c r="B187" s="220"/>
-      <c r="C187" s="382"/>
-      <c r="D187" s="383"/>
-      <c r="E187" s="383"/>
-      <c r="F187" s="384"/>
+      <c r="C187" s="227"/>
+      <c r="D187" s="227"/>
+      <c r="E187" s="227"/>
+      <c r="F187" s="227"/>
       <c r="G187" s="227"/>
       <c r="H187" s="227"/>
       <c r="I187" s="227"/>
@@ -18453,13 +18453,13 @@
     <row r="188" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A188" s="240"/>
       <c r="B188" s="220"/>
-      <c r="C188" s="261"/>
+      <c r="C188" s="227"/>
       <c r="D188" s="385"/>
       <c r="E188" s="385"/>
       <c r="F188" s="385"/>
       <c r="G188" s="218"/>
-      <c r="H188" s="253"/>
-      <c r="I188" s="253"/>
+      <c r="H188" s="227"/>
+      <c r="I188" s="227"/>
       <c r="J188" s="220"/>
       <c r="K188" s="220"/>
       <c r="L188" s="227"/>
@@ -18509,10 +18509,10 @@
     <row r="190" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A190" s="255"/>
       <c r="B190" s="220"/>
-      <c r="C190" s="382"/>
-      <c r="D190" s="383"/>
-      <c r="E190" s="383"/>
-      <c r="F190" s="384"/>
+      <c r="C190" s="227"/>
+      <c r="D190" s="227"/>
+      <c r="E190" s="227"/>
+      <c r="F190" s="227"/>
       <c r="G190" s="227"/>
       <c r="H190" s="227"/>
       <c r="I190" s="227"/>
@@ -18867,13 +18867,13 @@
     <row r="201" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A201" s="240"/>
       <c r="B201" s="220"/>
-      <c r="C201" s="217"/>
-      <c r="D201" s="356"/>
-      <c r="E201" s="357"/>
-      <c r="F201" s="358"/>
+      <c r="C201" s="227"/>
+      <c r="D201" s="227"/>
+      <c r="E201" s="227"/>
+      <c r="F201" s="227"/>
       <c r="G201" s="218"/>
-      <c r="H201" s="219"/>
-      <c r="I201" s="219"/>
+      <c r="H201" s="227"/>
+      <c r="I201" s="227"/>
       <c r="J201" s="220"/>
       <c r="K201" s="220"/>
       <c r="L201" s="236">
@@ -19013,13 +19013,13 @@
     <row r="206" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A206" s="240"/>
       <c r="B206" s="220"/>
-      <c r="C206" s="217"/>
-      <c r="D206" s="356"/>
-      <c r="E206" s="357"/>
-      <c r="F206" s="358"/>
+      <c r="C206" s="227"/>
+      <c r="D206" s="227"/>
+      <c r="E206" s="227"/>
+      <c r="F206" s="227"/>
       <c r="G206" s="218"/>
-      <c r="H206" s="219"/>
-      <c r="I206" s="219"/>
+      <c r="H206" s="227"/>
+      <c r="I206" s="227"/>
       <c r="J206" s="220"/>
       <c r="K206" s="220"/>
       <c r="L206" s="236">

</xml_diff>

<commit_message>
SE Full!G1's filing deadline follows the tax year, not a fixed 2027
The banner used to print a hardcoded "by 31st January 2027" regardless of
which year the package was generated for. The cell now reads a formula
concatenating the static wording with TEXT(Admin!B21,"yyyy") -- B21 is
already the online filing deadline (always 31 January, two years after the
tax year's start), used elsewhere on the Income Tax sheet's "Amounts
Payable by" line. The generator rolls G1's cached value alongside the
other Admin echoes (Q2, V2, G141) so a package opened without recalculating
still shows the right year, and the calculator engine mirrors the same
formula so both engines agree.

Two checks anchor the fix to the scenario's own tax year end rather than to
the sheet's own Admin echo: one on Admin!B21 itself, one on the SE Full
banner text. Both are proven breakable by JSZip cell corruption.
</commit_message>
<xml_diff>
--- a/app/templates/se/Financialaccounts.xlsx
+++ b/app/templates/se/Financialaccounts.xlsx
@@ -12739,8 +12739,9 @@
       <c r="D1" s="334"/>
       <c r="E1" s="334"/>
       <c r="F1" s="334"/>
-      <c r="G1" s="335" t="s">
-        <v>438</v>
+      <c r="G1" s="335" t="str">
+        <f>"COPY DETAILS TO HMRC FORM          Submit HMRC RETURN ONLINE                   by 31st January "&amp;TEXT(Admin!B21,"yyyy")</f>
+        <v>COPY DETAILS TO HMRC FORM          Submit HMRC RETURN ONLINE                   by 31st January 2027</v>
       </c>
       <c r="H1" s="336"/>
       <c r="I1" s="336"/>

</xml_diff>